<commit_message>
NER local de l'extension A1, réhydratation des jetons et réglages de détection
- API : nouveau module /v1/models/ner qui sert le modèle NER de l'extension
  avec vérification SHA-256 (empreintes figées dans @acg/shared) ;
  script pnpm models:ner pour déposer le modèle sur le serveur.
- Extension A1 : NER exécuté dans un document offscreen, récupération du
  modèle via l'API puis Hugging Face en repli ; réhydratation locale des
  jetons dans un Shadow DOM fermé, sans toucher la page du service d'IA.
- Detection Engine : réglages post-détection (seuils, bonus de contexte,
  listes d'autorisation), règles téléphone dédiées, masquage revu.
- Agent runtime : tests des liaisons de jetons et des actions sur fixtures.
- Fixtures fichiers régénérées, guide opérationnel A2, README et .env.example.
</commit_message>
<xml_diff>
--- a/data/fixtures-fichiers/09-MASK-cotisations.xlsx
+++ b/data/fixtures-fichiers/09-MASK-cotisations.xlsx
@@ -4,6 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Cotisations" sheetId="1" r:id="rId1"/>
+    <sheet name="Relances" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,9 +408,12 @@
         <v>N° employeur</v>
       </c>
       <c r="C1" t="str">
-        <v>Montant cotisations FCFA</v>
+        <v>Période</v>
       </c>
       <c r="D1" t="str">
+        <v>Montant dû</v>
+      </c>
+      <c r="E1" t="str">
         <v>Contact</v>
       </c>
     </row>
@@ -421,9 +425,12 @@
         <v>employeur cnss E4455667</v>
       </c>
       <c r="C2" t="str">
+        <v>T1</v>
+      </c>
+      <c r="D2" t="str">
         <v>15 000 000 FCFA</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>finance@demo.bj</v>
       </c>
     </row>
@@ -435,15 +442,96 @@
         <v>employeur cnss E1122334</v>
       </c>
       <c r="C3" t="str">
+        <v>T1</v>
+      </c>
+      <c r="D3" t="str">
         <v>3 200 000 FCFA</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>paie@test.bj</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>ETS Exemple</v>
+      </c>
+      <c r="B4" t="str">
+        <v>employeur cnss E9988776</v>
+      </c>
+      <c r="C4" t="str">
+        <v>T1</v>
+      </c>
+      <c r="D4" t="str">
+        <v>740 000 FCFA</v>
+      </c>
+      <c r="E4" t="str">
+        <v>rh@exemple.bj</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>SA Fictive</v>
+      </c>
+      <c r="B5" t="str">
+        <v>employeur cnss E5566778</v>
+      </c>
+      <c r="C5" t="str">
+        <v>T1</v>
+      </c>
+      <c r="D5" t="str">
+        <v>9 150 000 FCFA</v>
+      </c>
+      <c r="E5" t="str">
+        <v>compta@fictive.bj</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>N° employeur</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Relance</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Montant restant</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>employeur cnss E1122334</v>
+      </c>
+      <c r="B2" t="str">
+        <v>1re relance</v>
+      </c>
+      <c r="C2" t="str">
+        <v>1 600 000 FCFA</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>employeur cnss E9988776</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Mise en demeure</v>
+      </c>
+      <c r="C3" t="str">
+        <v>740 000 FCFA</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>